<commit_message>
add ciclos.py to demonstrate list iteration in Python
</commit_message>
<xml_diff>
--- a/sesion-3/pandas/lectura_archivo/data_ventas_enero_xlsx.xlsx
+++ b/sesion-3/pandas/lectura_archivo/data_ventas_enero_xlsx.xlsx
@@ -5,15 +5,16 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hpveg\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hpveg\Documents\idat-grupo-7\sesion-3\pandas\lectura_archivo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89712DB7-EB0B-4486-A0CA-D64A429E8658}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F80DB27-3456-4D0E-AE07-B90DB9FB7420}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Hoja1" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
   <si>
     <t>id_venta</t>
   </si>
@@ -46,6 +47,24 @@
   </si>
   <si>
     <t>Ana</t>
+  </si>
+  <si>
+    <t>Nombres</t>
+  </si>
+  <si>
+    <t>Edades</t>
+  </si>
+  <si>
+    <t>Pais</t>
+  </si>
+  <si>
+    <t>Juan</t>
+  </si>
+  <si>
+    <t>Peru</t>
+  </si>
+  <si>
+    <t>Nicol</t>
   </si>
 </sst>
 </file>
@@ -88,9 +107,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -383,19 +401,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
     </row>
@@ -414,6 +432,49 @@
       </c>
       <c r="E2" t="s">
         <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{873CCD89-4A73-4102-BD89-5CB6C9C50652}">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2">
+        <v>20</v>
+      </c>
+      <c r="C2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3">
+        <v>30</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>